<commit_message>
empty fields + some updates
</commit_message>
<xml_diff>
--- a/import/data_import/PNC00003 PET DASB collection/PN000017 CIMBI1/PublicnEUro_PN000017.xlsx
+++ b/import/data_import/PNC00003 PET DASB collection/PN000017 CIMBI1/PublicnEUro_PN000017.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PublicnEUro\DataCatalogue\import\data_import\PNC00003 PET DASB collection\PN000017 CIMBI1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FC687F8-9047-4A84-ADEE-5636EF470A52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D547D51-05C5-426F-AC26-94900896F623}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10560" tabRatio="599" firstSheet="2" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10560" tabRatio="599" firstSheet="1" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="dataset_info" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="79">
   <si>
     <t># bold fields are required</t>
   </si>
@@ -258,9 +258,6 @@
     <t>Content</t>
   </si>
   <si>
-    <t>UCBJ, PET, T1w, T2w, SV2A, 11C, dynamic</t>
-  </si>
-  <si>
     <t>PN000012</t>
   </si>
   <si>
@@ -268,15 +265,6 @@
   </si>
   <si>
     <t>Age range [min max]</t>
-  </si>
-  <si>
-    <t>[20 83]</t>
-  </si>
-  <si>
-    <t>PET UCB-J in healthy adult participants across the life span</t>
-  </si>
-  <si>
-    <t>The dataset contains 120 min dynamic scan starting with C11-UCBJ bolus along with T1w and T2w MRI data from people aged between 20 and 83 years old.</t>
   </si>
   <si>
     <t>Peter.Steen.Jensen@nru.dk</t>
@@ -298,30 +286,6 @@
 7. GENERAL PROVISIONS. 7.1 Governing law. This Agreement shall be governed in accordance with Danish Law. Each Party submits to the exclusive jurisdiction of the courts of Copenhagen, Denmark. 7.2 Relationship of the Parties. This Agreement does not create a partnership, agency, fiduciary or other relationship, except the relationship of contracting parties. A Party shall not represent that another Party or any of their staff in any way endorse, support or approve of, any products, services, Intellectual Property or business of the representing party unless that other Party has given its express written consent to such representation. 7.3 Entire agreement. This DUA constitutes the entire agreement of the Parties with respect to its subject matter and supersedes all prior oral or written representations and agreements. 7.4 Variation. This DUA may only be varied in writing signed by the Parties. 7.5 Assignment. The receiving data controller must not assign its rights under this DUA. 7.6 Waiver. A Party's failure to exercise or delay in exercising a right, power or remedy does not operate as a waiver of that right, power or remedy and does not preclude the future exercise of that right, power or remedy. To be effective, a waiver of a right, power or remedy must be in writing and signed by the Party granting the waiver. 7.7 Severance. If any provision or part provision of this DUA is invalid or unenforceable, such provision shall be deemed deleted but only to the extent necessary and the remaining provisions of this Agreement shall remain in full force and effect. 7.8 Force Majeure. A Party to this Agreement shall not be responsible or liable for any non-performance or delay in performance of any of its obligations under this Agreement that is caused by an act or event that is beyond the reasonable control of that Party ('Force Majeure Event'), provided that it promptly notifies the other parties (with appropriate details); and takes all reasonable steps to work around or reduce the effects of the Force Majeure Event. 7.9 Obligations. Each Party's obligations and liabilities under this Agreement are several and not joint or joint and several.</t>
   </si>
   <si>
-    <t>Sophia Armand</t>
-  </si>
-  <si>
-    <t>Gitte Moos Knudsen</t>
-  </si>
-  <si>
-    <t>Annette Johansen</t>
-  </si>
-  <si>
-    <t>Gitte.Knudsen@nru.dk</t>
-  </si>
-  <si>
-    <t>https://orcid.org/0000-0003-0264-2368</t>
-  </si>
-  <si>
-    <t>soa@psy.ku.dk</t>
-  </si>
-  <si>
-    <t>https://orcid.org/0000-0001-6368-3329</t>
-  </si>
-  <si>
-    <t>https://orcid.org/0000-0003-1508-6866</t>
-  </si>
-  <si>
     <t>Cyril Pernet</t>
   </si>
   <si>
@@ -329,12 +293,6 @@
   </si>
   <si>
     <t>Neurobiology Researh Unit</t>
-  </si>
-  <si>
-    <t>R281-2018-131</t>
-  </si>
-  <si>
-    <t>Lundbeck Foundation</t>
   </si>
   <si>
     <t>Martin Nørgaard</t>
@@ -1054,6 +1012,9 @@
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1089,9 +1050,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1318,20 +1276,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A1" s="85" t="s">
+      <c r="A1" s="86" t="s">
         <v>31</v>
       </c>
-      <c r="B1" s="87" t="s">
+      <c r="B1" s="88" t="s">
         <v>41</v>
       </c>
-      <c r="C1" s="89" t="s">
+      <c r="C1" s="90" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="2" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="86"/>
-      <c r="B2" s="88"/>
-      <c r="C2" s="90"/>
+      <c r="A2" s="87"/>
+      <c r="B2" s="89"/>
+      <c r="C2" s="91"/>
     </row>
     <row r="3" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A3" s="15" t="s">
@@ -1340,9 +1298,7 @@
       <c r="B3" s="47" t="s">
         <v>42</v>
       </c>
-      <c r="C3" s="52" t="s">
-        <v>74</v>
-      </c>
+      <c r="C3" s="52"/>
     </row>
     <row r="4" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A4" s="15" t="s">
@@ -1351,9 +1307,7 @@
       <c r="B4" s="60" t="s">
         <v>40</v>
       </c>
-      <c r="C4" s="53" t="s">
-        <v>75</v>
-      </c>
+      <c r="C4" s="53"/>
     </row>
     <row r="5" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A5" s="15" t="s">
@@ -1362,9 +1316,7 @@
       <c r="B5" s="48" t="s">
         <v>45</v>
       </c>
-      <c r="C5" s="53" t="s">
-        <v>69</v>
-      </c>
+      <c r="C5" s="53"/>
     </row>
     <row r="6" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A6" s="15" t="s">
@@ -1379,7 +1331,7 @@
       <c r="A7" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="B7" s="93" t="s">
+      <c r="B7" s="94" t="s">
         <v>32</v>
       </c>
       <c r="C7" s="53" t="s">
@@ -1390,7 +1342,7 @@
       <c r="A8" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="94"/>
+      <c r="B8" s="95"/>
       <c r="C8" s="78">
         <v>4.8622685185185185E-2</v>
       </c>
@@ -1421,7 +1373,7 @@
       <c r="A11" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="B11" s="91" t="s">
+      <c r="B11" s="92" t="s">
         <v>22</v>
       </c>
       <c r="C11" s="13"/>
@@ -1447,7 +1399,7 @@
       <c r="A12" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="B12" s="92"/>
+      <c r="B12" s="93"/>
       <c r="C12" s="14"/>
       <c r="D12" s="3"/>
       <c r="E12" s="3"/>
@@ -1471,7 +1423,7 @@
       <c r="A13" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="B13" s="91" t="s">
+      <c r="B13" s="92" t="s">
         <v>29</v>
       </c>
       <c r="C13" s="14"/>
@@ -1497,7 +1449,7 @@
       <c r="A14" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="B14" s="92"/>
+      <c r="B14" s="93"/>
       <c r="C14" s="14"/>
       <c r="D14" s="3"/>
       <c r="E14" s="3"/>
@@ -1617,7 +1569,7 @@
         <v>55</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="23" spans="1:20" x14ac:dyDescent="0.35">
@@ -1628,7 +1580,7 @@
         <v>56</v>
       </c>
       <c r="C23" s="73" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
   </sheetData>
@@ -1672,25 +1624,19 @@
       <c r="A2" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B2" s="8">
-        <v>41</v>
-      </c>
+      <c r="B2" s="8"/>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="27" t="s">
         <v>33</v>
       </c>
-      <c r="B3" s="8">
-        <v>15</v>
-      </c>
+      <c r="B3" s="8"/>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="B4" s="8">
-        <v>26</v>
-      </c>
+      <c r="B4" s="8"/>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" s="8" t="s">
@@ -1702,25 +1648,19 @@
       <c r="A6" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="8">
-        <v>41</v>
-      </c>
+      <c r="B6" s="8"/>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="8">
-        <v>0</v>
-      </c>
+      <c r="B7" s="8"/>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" s="79" t="s">
-        <v>72</v>
-      </c>
-      <c r="B8" s="79" t="s">
-        <v>73</v>
-      </c>
+        <v>71</v>
+      </c>
+      <c r="B8" s="79"/>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" s="49"/>
@@ -1764,7 +1704,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="80" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
@@ -1774,7 +1714,7 @@
         <v>6</v>
       </c>
       <c r="B4" s="61" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="C4" s="1"/>
     </row>
@@ -2817,72 +2757,72 @@
       <c r="A3" s="76" t="s">
         <v>63</v>
       </c>
-      <c r="B3" s="95" t="s">
-        <v>78</v>
+      <c r="B3" s="96" t="s">
+        <v>74</v>
       </c>
       <c r="D3" s="75" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="16" x14ac:dyDescent="0.45">
-      <c r="B4" s="96"/>
+      <c r="B4" s="97"/>
       <c r="D4" s="77" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B5" s="96"/>
+      <c r="B5" s="97"/>
       <c r="D5" s="75" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="16" x14ac:dyDescent="0.45">
-      <c r="B6" s="96"/>
+      <c r="B6" s="97"/>
       <c r="D6" s="77" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B7" s="96"/>
+      <c r="B7" s="97"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B8" s="96"/>
+      <c r="B8" s="97"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B9" s="96"/>
+      <c r="B9" s="97"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B10" s="96"/>
+      <c r="B10" s="97"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B11" s="96"/>
+      <c r="B11" s="97"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B12" s="96"/>
+      <c r="B12" s="97"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B13" s="96"/>
+      <c r="B13" s="97"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B14" s="96"/>
+      <c r="B14" s="97"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B15" s="96"/>
+      <c r="B15" s="97"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B16" s="96"/>
+      <c r="B16" s="97"/>
     </row>
     <row r="17" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B17" s="96"/>
+      <c r="B17" s="97"/>
     </row>
     <row r="18" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B18" s="96"/>
+      <c r="B18" s="97"/>
     </row>
     <row r="19" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B19" s="96"/>
+      <c r="B19" s="97"/>
     </row>
     <row r="20" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B20" s="96"/>
+      <c r="B20" s="97"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2933,37 +2873,21 @@
       <c r="D3" s="1"/>
     </row>
     <row r="4" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="81" t="s">
-        <v>79</v>
-      </c>
-      <c r="B4" s="82" t="s">
-        <v>84</v>
-      </c>
-      <c r="C4" s="63" t="s">
-        <v>85</v>
-      </c>
+      <c r="A4" s="81"/>
+      <c r="B4" s="82"/>
+      <c r="C4" s="63"/>
       <c r="D4" s="1"/>
     </row>
     <row r="5" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="30" t="s">
-        <v>80</v>
-      </c>
-      <c r="B5" s="62" t="s">
-        <v>82</v>
-      </c>
-      <c r="C5" s="63" t="s">
-        <v>86</v>
-      </c>
+      <c r="A5" s="30"/>
+      <c r="B5" s="62"/>
+      <c r="C5" s="63"/>
       <c r="D5" s="1"/>
     </row>
     <row r="6" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="81" t="s">
-        <v>81</v>
-      </c>
+      <c r="A6" s="81"/>
       <c r="B6" s="62"/>
-      <c r="C6" s="82" t="s">
-        <v>83</v>
-      </c>
+      <c r="C6" s="82"/>
       <c r="D6" s="1"/>
     </row>
     <row r="7" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
@@ -3975,11 +3899,6 @@
   </sheetData>
   <hyperlinks>
     <hyperlink ref="C3" r:id="rId1" display="https://orcid.org/" xr:uid="{936A8A87-9477-4811-BF8F-5F0EE214B672}"/>
-    <hyperlink ref="B5" r:id="rId2" xr:uid="{320DC7AD-ED03-4B72-B19C-26AB38411C3B}"/>
-    <hyperlink ref="C6" r:id="rId3" tooltip="Orcid" xr:uid="{50599A43-BC42-460E-859B-3062BD989B6A}"/>
-    <hyperlink ref="B4" r:id="rId4" display="https://psychology.ku.dk/staff/academic_staff/?pure=en/persons/524413" xr:uid="{C6ED1BD2-C877-4842-A746-DF0BFDD2FDE0}"/>
-    <hyperlink ref="C4" r:id="rId5" xr:uid="{93740643-E2D0-427C-B036-EC3936E91360}"/>
-    <hyperlink ref="C5" r:id="rId6" xr:uid="{7734ACE8-B15D-49F1-B59D-C0604088D307}"/>
   </hyperlinks>
   <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait"/>
@@ -4015,26 +3934,26 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" s="81" t="s">
-        <v>87</v>
+        <v>75</v>
       </c>
       <c r="B4" s="83" t="s">
-        <v>89</v>
+        <v>77</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" s="81" t="s">
-        <v>88</v>
+        <v>76</v>
       </c>
       <c r="B5" s="83" t="s">
-        <v>89</v>
+        <v>77</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A6" s="97" t="s">
-        <v>92</v>
+      <c r="A6" s="85" t="s">
+        <v>78</v>
       </c>
       <c r="B6" s="83" t="s">
-        <v>89</v>
+        <v>77</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
@@ -4090,12 +4009,8 @@
       </c>
     </row>
     <row r="4" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="84" t="s">
-        <v>91</v>
-      </c>
-      <c r="B4" s="36" t="s">
-        <v>90</v>
-      </c>
+      <c r="A4" s="84"/>
+      <c r="B4" s="36"/>
       <c r="C4" s="37"/>
     </row>
     <row r="5" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">

</xml_diff>